<commit_message>
fix: xdb upload on_exists=ERROR log is now assigned to each existing instance (#331)
Co-authored-by: Ivo van Walle <ivo.van.walle@rivm.nl>
Co-authored-by: Sander Sluis <sander@specto.nl>
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_upload/test_casedb_case_upload.xlsx
+++ b/test/casedb/integration/case_upload/test_casedb_case_upload.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05BBC205-3CB8-4821-B304-8186431C4FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CECEE2A4-2126-4F29-8A4C-434B96B9F08E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" firstSheet="7" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" firstSheet="20" activeTab="32" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ConceptSet" sheetId="30" r:id="rId1"/>
@@ -49,11 +49,6 @@
     <sheet name="UserShareCasePolicy" sheetId="23" r:id="rId34"/>
     <sheet name="OrganizationShareCasePolicy" sheetId="22" r:id="rId35"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId36"/>
-    <externalReference r:id="rId37"/>
-    <externalReference r:id="rId38"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">_CaseContentData!$A$1:$R$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">_CaseData!$A$1:$A$33</definedName>
@@ -4227,252 +4222,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="case.case_type"/>
-      <sheetName val="case.dim"/>
-      <sheetName val="case.col"/>
-      <sheetName val="case.case_type_dim"/>
-      <sheetName val="case.case_type_col"/>
-      <sheetName val="case.case_type_set_category"/>
-      <sheetName val="case.case_type_set"/>
-      <sheetName val="case.case_type_set_member"/>
-      <sheetName val="case.case_type_col_set"/>
-      <sheetName val="case.case_type_col_set_member"/>
-      <sheetName val="case.case"/>
-      <sheetName val="case.case_data_collection_link"/>
-      <sheetName val="case.case_set_category"/>
-      <sheetName val="case.case_set_status"/>
-      <sheetName val="case.case_set"/>
-      <sheetName val="case.case_set_member"/>
-      <sheetName val="case.case_set_data_collection_l"/>
-      <sheetName val="case.case.ACANTH"/>
-      <sheetName val="case.case.CRYP"/>
-      <sheetName val="case.case.ECHO"/>
-      <sheetName val="case.case.ECOLI"/>
-      <sheetName val="case.case.HEPA"/>
-      <sheetName val="case.case.MENI"/>
-      <sheetName val="case.case.MPOX"/>
-      <sheetName val="case.case.MRSA"/>
-      <sheetName val="case.case.NORO"/>
-      <sheetName val="case.case.PERT"/>
-      <sheetName val="case.case.SALM"/>
-      <sheetName val="case.case.SARS2"/>
-      <sheetName val="case.case.TUBE"/>
-      <sheetName val="case.case.YERS"/>
-      <sheetName val="case.tree_algorithm_class"/>
-      <sheetName val="case.tree_algorithm"/>
-      <sheetName val="case.genetic_distance_protocol"/>
-      <sheetName val="geo.region_set.copy"/>
-      <sheetName val="ontology.concept_set.copy"/>
-      <sheetName val="ontology.disease.copy"/>
-      <sheetName val="ontology.etiological_agen.copy"/>
-      <sheetName val="organization.organization.copy"/>
-      <sheetName val="organization.data_collecti.copy"/>
-      <sheetName val="geo.region.copy"/>
-      <sheetName val="map.residence"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
-      <sheetData sheetId="16" refreshError="1"/>
-      <sheetData sheetId="17" refreshError="1"/>
-      <sheetData sheetId="18" refreshError="1"/>
-      <sheetData sheetId="19" refreshError="1"/>
-      <sheetData sheetId="20" refreshError="1"/>
-      <sheetData sheetId="21" refreshError="1"/>
-      <sheetData sheetId="22" refreshError="1"/>
-      <sheetData sheetId="23" refreshError="1"/>
-      <sheetData sheetId="24" refreshError="1"/>
-      <sheetData sheetId="25" refreshError="1"/>
-      <sheetData sheetId="26" refreshError="1"/>
-      <sheetData sheetId="27" refreshError="1"/>
-      <sheetData sheetId="28" refreshError="1"/>
-      <sheetData sheetId="29" refreshError="1"/>
-      <sheetData sheetId="30" refreshError="1"/>
-      <sheetData sheetId="31" refreshError="1"/>
-      <sheetData sheetId="32" refreshError="1"/>
-      <sheetData sheetId="33"/>
-      <sheetData sheetId="34" refreshError="1"/>
-      <sheetData sheetId="35" refreshError="1"/>
-      <sheetData sheetId="36" refreshError="1"/>
-      <sheetData sheetId="37" refreshError="1"/>
-      <sheetData sheetId="38" refreshError="1"/>
-      <sheetData sheetId="39" refreshError="1"/>
-      <sheetData sheetId="40" refreshError="1"/>
-      <sheetData sheetId="41" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="organization.organization_set"/>
-      <sheetName val="organization.organization"/>
-      <sheetName val="organization.user"/>
-      <sheetName val="organization.site"/>
-      <sheetName val="organization.contact"/>
-      <sheetName val="organization.data_collection_se"/>
-      <sheetName val="organization.data_collection"/>
-      <sheetName val="organization.identifier_issuer"/>
-      <sheetName val="organization.org_id_issuer_link"/>
-      <sheetName val="organization.external_identifie"/>
-      <sheetName val="geo.region.copy"/>
-      <sheetName val="_identity_provider"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="seq.alignment_protocol"/>
-      <sheetName val="seq.allele"/>
-      <sheetName val="seq.allele_alignment"/>
-      <sheetName val="seq.allele_profile"/>
-      <sheetName val="seq.assembly_protocol"/>
-      <sheetName val="seq.ast_measurement"/>
-      <sheetName val="seq.ast_prediction"/>
-      <sheetName val="seq.ast_protocol"/>
-      <sheetName val="seq.kmer_detection_protocol"/>
-      <sheetName val="seq.kmer_profile"/>
-      <sheetName val="seq.mlva_detection_protocol"/>
-      <sheetName val="seq.mlva_profile"/>
-      <sheetName val="seq.sequencing_protocol"/>
-      <sheetName val="seq.locus"/>
-      <sheetName val="seq.locus_detection_protocol"/>
-      <sheetName val="seq.locus_profile"/>
-      <sheetName val="seq.locus_set"/>
-      <sheetName val="seq.locus_code_map"/>
-      <sheetName val="seq.pcr_measurement"/>
-      <sheetName val="seq.pcr_protocol"/>
-      <sheetName val="seq.read_set"/>
-      <sheetName val="seq.ref_allele"/>
-      <sheetName val="seq.ref_seq"/>
-      <sheetName val="seq.ref_snp"/>
-      <sheetName val="seq.ref_snp_set"/>
-      <sheetName val="seq.ref_snp_set_member"/>
-      <sheetName val="seq.sample"/>
-      <sheetName val="seq.sample_data_collection_link"/>
-      <sheetName val="seq.sample_identifier"/>
-      <sheetName val="seq.seq"/>
-      <sheetName val="seq.seq_alignment"/>
-      <sheetName val="seq.seq_category"/>
-      <sheetName val="seq.seq_category_set"/>
-      <sheetName val="seq.seq_classification"/>
-      <sheetName val="seq.seq_classification_protocol"/>
-      <sheetName val="seq.seq_distance"/>
-      <sheetName val="seq.seq_distance_protocol"/>
-      <sheetName val="seq.seq_taxonomy"/>
-      <sheetName val="seq.snp_detection_protocol"/>
-      <sheetName val="seq.snp_profile"/>
-      <sheetName val="seq.taxon"/>
-      <sheetName val="seq.taxonomy_protocol"/>
-      <sheetName val="seq.taxon_set"/>
-      <sheetName val="seq.taxon_set_member"/>
-      <sheetName val="seq.tree_algorithm"/>
-      <sheetName val="seq.tree_algorithm_class"/>
-      <sheetName val="file.file.copy"/>
-      <sheetName val="organization.data_collecti.copy"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-      <sheetData sheetId="27"/>
-      <sheetData sheetId="28"/>
-      <sheetData sheetId="29"/>
-      <sheetData sheetId="30"/>
-      <sheetData sheetId="31"/>
-      <sheetData sheetId="32"/>
-      <sheetData sheetId="33"/>
-      <sheetData sheetId="34"/>
-      <sheetData sheetId="35"/>
-      <sheetData sheetId="36"/>
-      <sheetData sheetId="37"/>
-      <sheetData sheetId="38"/>
-      <sheetData sheetId="39"/>
-      <sheetData sheetId="40"/>
-      <sheetData sheetId="41"/>
-      <sheetData sheetId="42"/>
-      <sheetData sheetId="43"/>
-      <sheetData sheetId="44"/>
-      <sheetData sheetId="45"/>
-      <sheetData sheetId="46"/>
-      <sheetData sheetId="47"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -22826,7 +22575,7 @@
         <v>970</v>
       </c>
       <c r="G2" s="19" t="b">
-        <f>IF($F2="CREATE",$I2,IF($F2="CREATE_CASES",OR($I2,AND($K2,$L2,$O2,$P2,$AN2,AP2,$AU2,$AW2,$BB2,$BD2)),"TBD"))</f>
+        <f t="shared" ref="G2:G33" si="0">IF($F2="CREATE",$I2,IF($F2="CREATE_CASES",OR($I2,AND($K2,$L2,$O2,$P2,$AN2,AP2,$AU2,$AW2,$BB2,$BD2)),"TBD"))</f>
         <v>1</v>
       </c>
       <c r="H2" s="6" t="str">
@@ -23001,7 +22750,7 @@
         <v>970</v>
       </c>
       <c r="G3" s="19" t="b">
-        <f>IF($F3="CREATE",$I3,IF($F3="CREATE_CASES",OR($I3,AND($K3,$L3,$O3,$P3,$AN3,AP3,$AU3,$AW3,$BB3,$BD3)),"TBD"))</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H3" s="6" t="str">
@@ -23176,7 +22925,7 @@
         <v>970</v>
       </c>
       <c r="G4" s="19" t="b">
-        <f>IF($F4="CREATE",$I4,IF($F4="CREATE_CASES",OR($I4,AND($K4,$L4,$O4,$P4,$AN4,AP4,$AU4,$AW4,$BB4,$BD4)),"TBD"))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H4" s="6" t="str">
@@ -23351,7 +23100,7 @@
         <v>970</v>
       </c>
       <c r="G5" s="19" t="b">
-        <f>IF($F5="CREATE",$I5,IF($F5="CREATE_CASES",OR($I5,AND($K5,$L5,$O5,$P5,$AN5,AP5,$AU5,$AW5,$BB5,$BD5)),"TBD"))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H5" s="6" t="str">
@@ -23526,7 +23275,7 @@
         <v>970</v>
       </c>
       <c r="G6" s="19" t="b">
-        <f>IF($F6="CREATE",$I6,IF($F6="CREATE_CASES",OR($I6,AND($K6,$L6,$O6,$P6,$AN6,AP6,$AU6,$AW6,$BB6,$BD6)),"TBD"))</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H6" s="6" t="str">
@@ -23701,7 +23450,7 @@
         <v>982</v>
       </c>
       <c r="G7" s="19" t="b">
-        <f ca="1">IF($F7="CREATE",$I7,IF($F7="CREATE_CASES",OR($I7,AND($K7,$L7,$O7,$P7,$AN7,AP7,$AU7,$AW7,$BB7,$BD7)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>1</v>
       </c>
       <c r="H7" s="6" t="str">
@@ -23876,7 +23625,7 @@
         <v>982</v>
       </c>
       <c r="G8" s="19" t="b">
-        <f ca="1">IF($F8="CREATE",$I8,IF($F8="CREATE_CASES",OR($I8,AND($K8,$L8,$O8,$P8,$AN8,AP8,$AU8,$AW8,$BB8,$BD8)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>1</v>
       </c>
       <c r="H8" s="6" t="str">
@@ -23935,7 +23684,7 @@
       </c>
       <c r="V8" s="6" t="b">
         <f>AND(IF($AJ8="",TRUE,$T8=INDEX(CaseTypeCol!$B:$B,MATCH($AJ8,CaseTypeCol!$A:$A,0))),IF($AQ8="",TRUE,$T8=INDEX(CaseTypeCol!$B:$B,MATCH($AQ8,CaseTypeCol!$A:$A,0))),IF($AX8="",TRUE,$T8=INDEX(CaseTypeCol!$B:$B,MATCH($AX8,CaseTypeCol!$A:$A,0))))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X8" t="s">
         <v>11</v>
@@ -24003,22 +23752,22 @@
         <v>0</v>
       </c>
       <c r="AQ8" t="s">
-        <v>1181</v>
+        <v>1173</v>
       </c>
       <c r="AR8" t="s">
         <v>1185</v>
       </c>
       <c r="AS8" s="6" t="str">
         <f>IF($AQ8="","",INDEX(CaseTypeCol!$J:$J,MATCH($AQ8,CaseTypeCol!$A:$A,0)))</f>
-        <v>case_type_col2_19_0_1_GENETIC_READS</v>
+        <v>case_type_col1_19_0_1_GENETIC_READS</v>
       </c>
       <c r="AT8" s="6" t="b" cm="1">
         <f t="array" aca="1" ref="AT8" ca="1">IF($AQ8="",TRUE,IF($J8="",FALSE,IF(INDIRECT("OrganizationAccessCasePolicy!J"&amp;$J8)="",FALSE,NOT(ISNA(MATCH(INDIRECT("OrganizationAccessCasePolicy!J"&amp;$J8)&amp;"|"&amp;$AQ8,CaseTypeColSetMember!$H:$H,0))))))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU8" s="6" t="b" cm="1">
         <f t="array" aca="1" ref="AU8" ca="1">IF($AQ8="",TRUE,IF($J8="",FALSE,IF(INDIRECT("OrganizationAccessCasePolicy!L"&amp;$J8)="",FALSE,NOT(ISNA(MATCH(INDIRECT("OrganizationAccessCasePolicy!L"&amp;$J8)&amp;"|"&amp;$AQ8,CaseTypeColSetMember!$H:$H,0))))))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV8" s="6" t="b" cm="1">
         <f t="array" aca="1" ref="AV8" ca="1">IF($AQ8="",TRUE,IF($N8="",FALSE,IF(INDIRECT("UserAccessCasePolicy!I"&amp;$N8)="",FALSE,NOT(ISNA(MATCH(INDIRECT("UserAccessCasePolicy!I"&amp;$N8)&amp;"|"&amp;$AQ8,CaseTypeColSetMember!$H:$H,0))))))</f>
@@ -24070,7 +23819,7 @@
         <v>982</v>
       </c>
       <c r="G9" s="19" t="b">
-        <f ca="1">IF($F9="CREATE",$I9,IF($F9="CREATE_CASES",OR($I9,AND($K9,$L9,$O9,$P9,$AN9,AP9,$AU9,$AW9,$BB9,$BD9)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>1</v>
       </c>
       <c r="H9" s="6" t="str">
@@ -24245,7 +23994,7 @@
         <v>982</v>
       </c>
       <c r="G10" s="19" t="b">
-        <f ca="1">IF($F10="CREATE",$I10,IF($F10="CREATE_CASES",OR($I10,AND($K10,$L10,$O10,$P10,$AN10,AP10,$AU10,$AW10,$BB10,$BD10)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H10" s="6" t="str">
@@ -24420,7 +24169,7 @@
         <v>982</v>
       </c>
       <c r="G11" s="19" t="b">
-        <f ca="1">IF($F11="CREATE",$I11,IF($F11="CREATE_CASES",OR($I11,AND($K11,$L11,$O11,$P11,$AN11,AP11,$AU11,$AW11,$BB11,$BD11)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H11" s="6" t="str">
@@ -24595,7 +24344,7 @@
         <v>982</v>
       </c>
       <c r="G12" s="19" t="b">
-        <f ca="1">IF($F12="CREATE",$I12,IF($F12="CREATE_CASES",OR($I12,AND($K12,$L12,$O12,$P12,$AN12,AP12,$AU12,$AW12,$BB12,$BD12)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H12" s="6" t="str">
@@ -24770,7 +24519,7 @@
         <v>982</v>
       </c>
       <c r="G13" s="19" t="b">
-        <f ca="1">IF($F13="CREATE",$I13,IF($F13="CREATE_CASES",OR($I13,AND($K13,$L13,$O13,$P13,$AN13,AP13,$AU13,$AW13,$BB13,$BD13)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H13" s="6" t="str">
@@ -24945,7 +24694,7 @@
         <v>982</v>
       </c>
       <c r="G14" s="19" t="b">
-        <f ca="1">IF($F14="CREATE",$I14,IF($F14="CREATE_CASES",OR($I14,AND($K14,$L14,$O14,$P14,$AN14,AP14,$AU14,$AW14,$BB14,$BD14)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H14" s="6" t="str">
@@ -25120,7 +24869,7 @@
         <v>982</v>
       </c>
       <c r="G15" s="19" t="b">
-        <f ca="1">IF($F15="CREATE",$I15,IF($F15="CREATE_CASES",OR($I15,AND($K15,$L15,$O15,$P15,$AN15,AP15,$AU15,$AW15,$BB15,$BD15)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>1</v>
       </c>
       <c r="H15" s="6" t="str">
@@ -25295,7 +25044,7 @@
         <v>982</v>
       </c>
       <c r="G16" s="19" t="b">
-        <f ca="1">IF($F16="CREATE",$I16,IF($F16="CREATE_CASES",OR($I16,AND($K16,$L16,$O16,$P16,$AN16,AP16,$AU16,$AW16,$BB16,$BD16)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H16" s="6" t="str">
@@ -25470,7 +25219,7 @@
         <v>982</v>
       </c>
       <c r="G17" s="19" t="b">
-        <f ca="1">IF($F17="CREATE",$I17,IF($F17="CREATE_CASES",OR($I17,AND($K17,$L17,$O17,$P17,$AN17,AP17,$AU17,$AW17,$BB17,$BD17)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H17" s="6" t="str">
@@ -25645,7 +25394,7 @@
         <v>982</v>
       </c>
       <c r="G18" s="19" t="b">
-        <f ca="1">IF($F18="CREATE",$I18,IF($F18="CREATE_CASES",OR($I18,AND($K18,$L18,$O18,$P18,$AN18,AP18,$AU18,$AW18,$BB18,$BD18)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H18" s="6" t="str">
@@ -25820,7 +25569,7 @@
         <v>982</v>
       </c>
       <c r="G19" s="19" t="b">
-        <f ca="1">IF($F19="CREATE",$I19,IF($F19="CREATE_CASES",OR($I19,AND($K19,$L19,$O19,$P19,$AN19,AP19,$AU19,$AW19,$BB19,$BD19)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H19" s="6" t="str">
@@ -25995,7 +25744,7 @@
         <v>982</v>
       </c>
       <c r="G20" s="19" t="b">
-        <f ca="1">IF($F20="CREATE",$I20,IF($F20="CREATE_CASES",OR($I20,AND($K20,$L20,$O20,$P20,$AN20,AP20,$AU20,$AW20,$BB20,$BD20)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H20" s="6" t="str">
@@ -26170,7 +25919,7 @@
         <v>982</v>
       </c>
       <c r="G21" s="19" t="b">
-        <f ca="1">IF($F21="CREATE",$I21,IF($F21="CREATE_CASES",OR($I21,AND($K21,$L21,$O21,$P21,$AN21,AP21,$AU21,$AW21,$BB21,$BD21)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H21" s="6" t="str">
@@ -26345,7 +26094,7 @@
         <v>982</v>
       </c>
       <c r="G22" s="19" t="b">
-        <f ca="1">IF($F22="CREATE",$I22,IF($F22="CREATE_CASES",OR($I22,AND($K22,$L22,$O22,$P22,$AN22,AP22,$AU22,$AW22,$BB22,$BD22)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H22" s="6" t="str">
@@ -26520,7 +26269,7 @@
         <v>982</v>
       </c>
       <c r="G23" s="19" t="b">
-        <f ca="1">IF($F23="CREATE",$I23,IF($F23="CREATE_CASES",OR($I23,AND($K23,$L23,$O23,$P23,$AN23,AP23,$AU23,$AW23,$BB23,$BD23)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H23" s="6" t="str">
@@ -26695,7 +26444,7 @@
         <v>982</v>
       </c>
       <c r="G24" s="19" t="b">
-        <f ca="1">IF($F24="CREATE",$I24,IF($F24="CREATE_CASES",OR($I24,AND($K24,$L24,$O24,$P24,$AN24,AP24,$AU24,$AW24,$BB24,$BD24)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H24" s="6" t="str">
@@ -26870,7 +26619,7 @@
         <v>982</v>
       </c>
       <c r="G25" s="19" t="b">
-        <f ca="1">IF($F25="CREATE",$I25,IF($F25="CREATE_CASES",OR($I25,AND($K25,$L25,$O25,$P25,$AN25,AP25,$AU25,$AW25,$BB25,$BD25)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H25" s="6" t="str">
@@ -27045,7 +26794,7 @@
         <v>982</v>
       </c>
       <c r="G26" s="19" t="b">
-        <f ca="1">IF($F26="CREATE",$I26,IF($F26="CREATE_CASES",OR($I26,AND($K26,$L26,$O26,$P26,$AN26,AP26,$AU26,$AW26,$BB26,$BD26)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H26" s="6" t="str">
@@ -27220,7 +26969,7 @@
         <v>982</v>
       </c>
       <c r="G27" s="19" t="b">
-        <f ca="1">IF($F27="CREATE",$I27,IF($F27="CREATE_CASES",OR($I27,AND($K27,$L27,$O27,$P27,$AN27,AP27,$AU27,$AW27,$BB27,$BD27)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H27" s="6" t="str">
@@ -27395,7 +27144,7 @@
         <v>982</v>
       </c>
       <c r="G28" s="19" t="b">
-        <f ca="1">IF($F28="CREATE",$I28,IF($F28="CREATE_CASES",OR($I28,AND($K28,$L28,$O28,$P28,$AN28,AP28,$AU28,$AW28,$BB28,$BD28)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H28" s="6" t="str">
@@ -27570,7 +27319,7 @@
         <v>982</v>
       </c>
       <c r="G29" s="19" t="b">
-        <f ca="1">IF($F29="CREATE",$I29,IF($F29="CREATE_CASES",OR($I29,AND($K29,$L29,$O29,$P29,$AN29,AP29,$AU29,$AW29,$BB29,$BD29)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H29" s="6" t="str">
@@ -27745,7 +27494,7 @@
         <v>982</v>
       </c>
       <c r="G30" s="19" t="b">
-        <f ca="1">IF($F30="CREATE",$I30,IF($F30="CREATE_CASES",OR($I30,AND($K30,$L30,$O30,$P30,$AN30,AP30,$AU30,$AW30,$BB30,$BD30)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H30" s="6" t="str">
@@ -27920,7 +27669,7 @@
         <v>982</v>
       </c>
       <c r="G31" s="19" t="b">
-        <f ca="1">IF($F31="CREATE",$I31,IF($F31="CREATE_CASES",OR($I31,AND($K31,$L31,$O31,$P31,$AN31,AP31,$AU31,$AW31,$BB31,$BD31)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H31" s="6" t="str">
@@ -28095,7 +27844,7 @@
         <v>982</v>
       </c>
       <c r="G32" s="19" t="b">
-        <f ca="1">IF($F32="CREATE",$I32,IF($F32="CREATE_CASES",OR($I32,AND($K32,$L32,$O32,$P32,$AN32,AP32,$AU32,$AW32,$BB32,$BD32)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H32" s="6" t="str">
@@ -28270,7 +28019,7 @@
         <v>982</v>
       </c>
       <c r="G33" s="19" t="b">
-        <f ca="1">IF($F33="CREATE",$I33,IF($F33="CREATE_CASES",OR($I33,AND($K33,$L33,$O33,$P33,$AN33,AP33,$AU33,$AW33,$BB33,$BD33)),"TBD"))</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="H33" s="6" t="str">
@@ -28445,7 +28194,7 @@
         <v>982</v>
       </c>
       <c r="G34" s="19" t="b">
-        <f ca="1">IF($F34="CREATE",$I34,IF($F34="CREATE_CASES",OR($I34,AND($K34,$L34,$O34,$P34,$AN34,AP34,$AU34,$AW34,$BB34,$BD34)),"TBD"))</f>
+        <f t="shared" ref="G34:G65" ca="1" si="1">IF($F34="CREATE",$I34,IF($F34="CREATE_CASES",OR($I34,AND($K34,$L34,$O34,$P34,$AN34,AP34,$AU34,$AW34,$BB34,$BD34)),"TBD"))</f>
         <v>0</v>
       </c>
       <c r="H34" s="6" t="str">
@@ -28620,7 +28369,7 @@
         <v>982</v>
       </c>
       <c r="G35" s="19" t="b">
-        <f ca="1">IF($F35="CREATE",$I35,IF($F35="CREATE_CASES",OR($I35,AND($K35,$L35,$O35,$P35,$AN35,AP35,$AU35,$AW35,$BB35,$BD35)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H35" s="6" t="str">
@@ -28801,7 +28550,7 @@
         <v>982</v>
       </c>
       <c r="G36" s="19" t="b">
-        <f ca="1">IF($F36="CREATE",$I36,IF($F36="CREATE_CASES",OR($I36,AND($K36,$L36,$O36,$P36,$AN36,AP36,$AU36,$AW36,$BB36,$BD36)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H36" s="6" t="str">
@@ -28977,7 +28726,7 @@
         <v>982</v>
       </c>
       <c r="G37" s="19" t="b">
-        <f ca="1">IF($F37="CREATE",$I37,IF($F37="CREATE_CASES",OR($I37,AND($K37,$L37,$O37,$P37,$AN37,AP37,$AU37,$AW37,$BB37,$BD37)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H37" s="6" t="str">
@@ -29153,7 +28902,7 @@
         <v>982</v>
       </c>
       <c r="G38" s="19" t="b">
-        <f ca="1">IF($F38="CREATE",$I38,IF($F38="CREATE_CASES",OR($I38,AND($K38,$L38,$O38,$P38,$AN38,AP38,$AU38,$AW38,$BB38,$BD38)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H38" s="6" t="str">
@@ -29328,7 +29077,7 @@
         <v>982</v>
       </c>
       <c r="G39" s="19" t="b">
-        <f ca="1">IF($F39="CREATE",$I39,IF($F39="CREATE_CASES",OR($I39,AND($K39,$L39,$O39,$P39,$AN39,AP39,$AU39,$AW39,$BB39,$BD39)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H39" s="6" t="str">
@@ -29503,7 +29252,7 @@
         <v>982</v>
       </c>
       <c r="G40" s="19" t="b">
-        <f ca="1">IF($F40="CREATE",$I40,IF($F40="CREATE_CASES",OR($I40,AND($K40,$L40,$O40,$P40,$AN40,AP40,$AU40,$AW40,$BB40,$BD40)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H40" s="6" t="str">
@@ -29678,7 +29427,7 @@
         <v>982</v>
       </c>
       <c r="G41" s="19" t="b">
-        <f ca="1">IF($F41="CREATE",$I41,IF($F41="CREATE_CASES",OR($I41,AND($K41,$L41,$O41,$P41,$AN41,AP41,$AU41,$AW41,$BB41,$BD41)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H41" s="6" t="str">
@@ -29853,7 +29602,7 @@
         <v>982</v>
       </c>
       <c r="G42" s="19" t="b">
-        <f ca="1">IF($F42="CREATE",$I42,IF($F42="CREATE_CASES",OR($I42,AND($K42,$L42,$O42,$P42,$AN42,AP42,$AU42,$AW42,$BB42,$BD42)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H42" s="6" t="str">
@@ -30028,7 +29777,7 @@
         <v>982</v>
       </c>
       <c r="G43" s="19" t="b">
-        <f ca="1">IF($F43="CREATE",$I43,IF($F43="CREATE_CASES",OR($I43,AND($K43,$L43,$O43,$P43,$AN43,AP43,$AU43,$AW43,$BB43,$BD43)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H43" s="6" t="str">
@@ -30203,7 +29952,7 @@
         <v>982</v>
       </c>
       <c r="G44" s="19" t="b">
-        <f ca="1">IF($F44="CREATE",$I44,IF($F44="CREATE_CASES",OR($I44,AND($K44,$L44,$O44,$P44,$AN44,AP44,$AU44,$AW44,$BB44,$BD44)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H44" s="6" t="str">
@@ -30378,7 +30127,7 @@
         <v>982</v>
       </c>
       <c r="G45" s="19" t="b">
-        <f ca="1">IF($F45="CREATE",$I45,IF($F45="CREATE_CASES",OR($I45,AND($K45,$L45,$O45,$P45,$AN45,AP45,$AU45,$AW45,$BB45,$BD45)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H45" s="6" t="str">
@@ -30553,7 +30302,7 @@
         <v>982</v>
       </c>
       <c r="G46" s="19" t="b">
-        <f ca="1">IF($F46="CREATE",$I46,IF($F46="CREATE_CASES",OR($I46,AND($K46,$L46,$O46,$P46,$AN46,AP46,$AU46,$AW46,$BB46,$BD46)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H46" s="6" t="str">
@@ -30728,7 +30477,7 @@
         <v>982</v>
       </c>
       <c r="G47" s="19" t="b">
-        <f ca="1">IF($F47="CREATE",$I47,IF($F47="CREATE_CASES",OR($I47,AND($K47,$L47,$O47,$P47,$AN47,AP47,$AU47,$AW47,$BB47,$BD47)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H47" s="6" t="str">
@@ -30903,7 +30652,7 @@
         <v>982</v>
       </c>
       <c r="G48" s="19" t="b">
-        <f ca="1">IF($F48="CREATE",$I48,IF($F48="CREATE_CASES",OR($I48,AND($K48,$L48,$O48,$P48,$AN48,AP48,$AU48,$AW48,$BB48,$BD48)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H48" s="6" t="str">
@@ -31078,7 +30827,7 @@
         <v>982</v>
       </c>
       <c r="G49" s="19" t="b">
-        <f ca="1">IF($F49="CREATE",$I49,IF($F49="CREATE_CASES",OR($I49,AND($K49,$L49,$O49,$P49,$AN49,AP49,$AU49,$AW49,$BB49,$BD49)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H49" s="6" t="str">
@@ -31253,7 +31002,7 @@
         <v>982</v>
       </c>
       <c r="G50" s="19" t="b">
-        <f ca="1">IF($F50="CREATE",$I50,IF($F50="CREATE_CASES",OR($I50,AND($K50,$L50,$O50,$P50,$AN50,AP50,$AU50,$AW50,$BB50,$BD50)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H50" s="6" t="str">
@@ -31428,7 +31177,7 @@
         <v>982</v>
       </c>
       <c r="G51" s="19" t="b">
-        <f ca="1">IF($F51="CREATE",$I51,IF($F51="CREATE_CASES",OR($I51,AND($K51,$L51,$O51,$P51,$AN51,AP51,$AU51,$AW51,$BB51,$BD51)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H51" s="6" t="str">
@@ -31603,7 +31352,7 @@
         <v>982</v>
       </c>
       <c r="G52" s="19" t="b">
-        <f ca="1">IF($F52="CREATE",$I52,IF($F52="CREATE_CASES",OR($I52,AND($K52,$L52,$O52,$P52,$AN52,AP52,$AU52,$AW52,$BB52,$BD52)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H52" s="6" t="str">
@@ -31778,7 +31527,7 @@
         <v>982</v>
       </c>
       <c r="G53" s="19" t="b">
-        <f ca="1">IF($F53="CREATE",$I53,IF($F53="CREATE_CASES",OR($I53,AND($K53,$L53,$O53,$P53,$AN53,AP53,$AU53,$AW53,$BB53,$BD53)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H53" s="6" t="str">
@@ -31953,7 +31702,7 @@
         <v>982</v>
       </c>
       <c r="G54" s="19" t="b">
-        <f ca="1">IF($F54="CREATE",$I54,IF($F54="CREATE_CASES",OR($I54,AND($K54,$L54,$O54,$P54,$AN54,AP54,$AU54,$AW54,$BB54,$BD54)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H54" s="6" t="str">
@@ -32128,7 +31877,7 @@
         <v>982</v>
       </c>
       <c r="G55" s="19" t="b">
-        <f ca="1">IF($F55="CREATE",$I55,IF($F55="CREATE_CASES",OR($I55,AND($K55,$L55,$O55,$P55,$AN55,AP55,$AU55,$AW55,$BB55,$BD55)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H55" s="6" t="str">
@@ -32303,7 +32052,7 @@
         <v>982</v>
       </c>
       <c r="G56" s="19" t="b">
-        <f ca="1">IF($F56="CREATE",$I56,IF($F56="CREATE_CASES",OR($I56,AND($K56,$L56,$O56,$P56,$AN56,AP56,$AU56,$AW56,$BB56,$BD56)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H56" s="6" t="str">
@@ -32484,7 +32233,7 @@
         <v>982</v>
       </c>
       <c r="G57" s="19" t="b">
-        <f ca="1">IF($F57="CREATE",$I57,IF($F57="CREATE_CASES",OR($I57,AND($K57,$L57,$O57,$P57,$AN57,AP57,$AU57,$AW57,$BB57,$BD57)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H57" s="6" t="str">
@@ -32659,7 +32408,7 @@
         <v>982</v>
       </c>
       <c r="G58" s="19" t="b">
-        <f ca="1">IF($F58="CREATE",$I58,IF($F58="CREATE_CASES",OR($I58,AND($K58,$L58,$O58,$P58,$AN58,AP58,$AU58,$AW58,$BB58,$BD58)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H58" s="6" t="str">
@@ -32834,7 +32583,7 @@
         <v>982</v>
       </c>
       <c r="G59" s="19" t="b">
-        <f ca="1">IF($F59="CREATE",$I59,IF($F59="CREATE_CASES",OR($I59,AND($K59,$L59,$O59,$P59,$AN59,AP59,$AU59,$AW59,$BB59,$BD59)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H59" s="6" t="str">
@@ -33009,7 +32758,7 @@
         <v>982</v>
       </c>
       <c r="G60" s="19" t="b">
-        <f ca="1">IF($F60="CREATE",$I60,IF($F60="CREATE_CASES",OR($I60,AND($K60,$L60,$O60,$P60,$AN60,AP60,$AU60,$AW60,$BB60,$BD60)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H60" s="6" t="str">
@@ -33184,7 +32933,7 @@
         <v>982</v>
       </c>
       <c r="G61" s="19" t="b">
-        <f ca="1">IF($F61="CREATE",$I61,IF($F61="CREATE_CASES",OR($I61,AND($K61,$L61,$O61,$P61,$AN61,AP61,$AU61,$AW61,$BB61,$BD61)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H61" s="6" t="str">
@@ -33362,7 +33111,7 @@
         <v>982</v>
       </c>
       <c r="G62" s="19" t="b">
-        <f ca="1">IF($F62="CREATE",$I62,IF($F62="CREATE_CASES",OR($I62,AND($K62,$L62,$O62,$P62,$AN62,AP62,$AU62,$AW62,$BB62,$BD62)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H62" s="6" t="str">
@@ -33540,7 +33289,7 @@
         <v>982</v>
       </c>
       <c r="G63" s="19" t="b">
-        <f ca="1">IF($F63="CREATE",$I63,IF($F63="CREATE_CASES",OR($I63,AND($K63,$L63,$O63,$P63,$AN63,AP63,$AU63,$AW63,$BB63,$BD63)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H63" s="6" t="str">
@@ -33718,7 +33467,7 @@
         <v>982</v>
       </c>
       <c r="G64" s="19" t="b">
-        <f ca="1">IF($F64="CREATE",$I64,IF($F64="CREATE_CASES",OR($I64,AND($K64,$L64,$O64,$P64,$AN64,AP64,$AU64,$AW64,$BB64,$BD64)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H64" s="6" t="str">
@@ -33896,7 +33645,7 @@
         <v>982</v>
       </c>
       <c r="G65" s="19" t="b">
-        <f ca="1">IF($F65="CREATE",$I65,IF($F65="CREATE_CASES",OR($I65,AND($K65,$L65,$O65,$P65,$AN65,AP65,$AU65,$AW65,$BB65,$BD65)),"TBD"))</f>
+        <f t="shared" ca="1" si="1"/>
         <v>0</v>
       </c>
       <c r="H65" s="6" t="str">
@@ -34074,7 +33823,7 @@
         <v>982</v>
       </c>
       <c r="G66" s="19" t="b">
-        <f ca="1">IF($F66="CREATE",$I66,IF($F66="CREATE_CASES",OR($I66,AND($K66,$L66,$O66,$P66,$AN66,AP66,$AU66,$AW66,$BB66,$BD66)),"TBD"))</f>
+        <f t="shared" ref="G66:G76" ca="1" si="2">IF($F66="CREATE",$I66,IF($F66="CREATE_CASES",OR($I66,AND($K66,$L66,$O66,$P66,$AN66,AP66,$AU66,$AW66,$BB66,$BD66)),"TBD"))</f>
         <v>0</v>
       </c>
       <c r="H66" s="6" t="str">
@@ -34252,7 +34001,7 @@
         <v>982</v>
       </c>
       <c r="G67" s="19" t="b">
-        <f ca="1">IF($F67="CREATE",$I67,IF($F67="CREATE_CASES",OR($I67,AND($K67,$L67,$O67,$P67,$AN67,AP67,$AU67,$AW67,$BB67,$BD67)),"TBD"))</f>
+        <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
       <c r="H67" s="6" t="str">
@@ -34430,7 +34179,7 @@
         <v>982</v>
       </c>
       <c r="G68" s="19" t="b">
-        <f ca="1">IF($F68="CREATE",$I68,IF($F68="CREATE_CASES",OR($I68,AND($K68,$L68,$O68,$P68,$AN68,AP68,$AU68,$AW68,$BB68,$BD68)),"TBD"))</f>
+        <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
       <c r="H68" s="6" t="str">
@@ -34608,7 +34357,7 @@
         <v>982</v>
       </c>
       <c r="G69" s="19" t="b">
-        <f ca="1">IF($F69="CREATE",$I69,IF($F69="CREATE_CASES",OR($I69,AND($K69,$L69,$O69,$P69,$AN69,AP69,$AU69,$AW69,$BB69,$BD69)),"TBD"))</f>
+        <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
       <c r="H69" s="6" t="str">
@@ -34786,7 +34535,7 @@
         <v>982</v>
       </c>
       <c r="G70" s="19" t="b">
-        <f ca="1">IF($F70="CREATE",$I70,IF($F70="CREATE_CASES",OR($I70,AND($K70,$L70,$O70,$P70,$AN70,AP70,$AU70,$AW70,$BB70,$BD70)),"TBD"))</f>
+        <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
       <c r="H70" s="6" t="str">
@@ -34964,7 +34713,7 @@
         <v>982</v>
       </c>
       <c r="G71" s="19" t="b">
-        <f ca="1">IF($F71="CREATE",$I71,IF($F71="CREATE_CASES",OR($I71,AND($K71,$L71,$O71,$P71,$AN71,AP71,$AU71,$AW71,$BB71,$BD71)),"TBD"))</f>
+        <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
       <c r="H71" s="6" t="str">
@@ -35142,7 +34891,7 @@
         <v>982</v>
       </c>
       <c r="G72" s="19" t="b">
-        <f ca="1">IF($F72="CREATE",$I72,IF($F72="CREATE_CASES",OR($I72,AND($K72,$L72,$O72,$P72,$AN72,AP72,$AU72,$AW72,$BB72,$BD72)),"TBD"))</f>
+        <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
       <c r="H72" s="6" t="str">
@@ -35320,7 +35069,7 @@
         <v>982</v>
       </c>
       <c r="G73" s="19" t="b">
-        <f ca="1">IF($F73="CREATE",$I73,IF($F73="CREATE_CASES",OR($I73,AND($K73,$L73,$O73,$P73,$AN73,AP73,$AU73,$AW73,$BB73,$BD73)),"TBD"))</f>
+        <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
       <c r="H73" s="6" t="str">
@@ -35498,7 +35247,7 @@
         <v>982</v>
       </c>
       <c r="G74" s="19" t="b">
-        <f ca="1">IF($F74="CREATE",$I74,IF($F74="CREATE_CASES",OR($I74,AND($K74,$L74,$O74,$P74,$AN74,AP74,$AU74,$AW74,$BB74,$BD74)),"TBD"))</f>
+        <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
       <c r="H74" s="6" t="str">
@@ -35676,7 +35425,7 @@
         <v>982</v>
       </c>
       <c r="G75" s="19" t="b">
-        <f ca="1">IF($F75="CREATE",$I75,IF($F75="CREATE_CASES",OR($I75,AND($K75,$L75,$O75,$P75,$AN75,AP75,$AU75,$AW75,$BB75,$BD75)),"TBD"))</f>
+        <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
       <c r="H75" s="6" t="str">
@@ -35854,7 +35603,7 @@
         <v>982</v>
       </c>
       <c r="G76" s="19" t="b">
-        <f ca="1">IF($F76="CREATE",$I76,IF($F76="CREATE_CASES",OR($I76,AND($K76,$L76,$O76,$P76,$AN76,AP76,$AU76,$AW76,$BB76,$BD76)),"TBD"))</f>
+        <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
       <c r="H76" s="6" t="str">
@@ -41251,6 +41000,7 @@
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:H116"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -41290,7 +41040,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>571</v>
       </c>
@@ -41313,7 +41063,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-a221-af7e-774497e4801a</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>572</v>
       </c>
@@ -41336,7 +41086,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-ce42-568c-c8e8405533a1</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>573</v>
       </c>
@@ -41359,7 +41109,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-1062-3f54-74f967fd95da</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>574</v>
       </c>
@@ -41382,7 +41132,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-f372-ce25-38616e4c214d</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>575</v>
       </c>
@@ -41405,7 +41155,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-b8fc-9de5-72be815082e0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>576</v>
       </c>
@@ -41428,7 +41178,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-371a-179d-9c036f8c66f2</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>577</v>
       </c>
@@ -41451,7 +41201,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-7325-a3c3-0be3c6d6193b</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>578</v>
       </c>
@@ -41474,7 +41224,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-61b3-63f1-bc4f52741be3</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>579</v>
       </c>
@@ -41497,7 +41247,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-f6da-4821-571b2b52bd5b</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>580</v>
       </c>
@@ -41520,7 +41270,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-3dff-04fd-3c65614d655d</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>581</v>
       </c>
@@ -41543,7 +41293,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-c3d9-408d-20f86d523b9f</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>582</v>
       </c>
@@ -41566,7 +41316,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-e425-5793-c7c455726f56</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>583</v>
       </c>
@@ -41589,7 +41339,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-0bc5-2af0-dbe7f34bc5cc</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>584</v>
       </c>
@@ -41612,7 +41362,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-58d8-f78b-17d1fd52333b</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>585</v>
       </c>
@@ -41635,7 +41385,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-f61d-4edc-07bcd51c380d</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>586</v>
       </c>
@@ -41658,7 +41408,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-2afc-2c12-93e895132544</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>587</v>
       </c>
@@ -41681,7 +41431,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-c453-7e15-c4a877df12b1</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>588</v>
       </c>
@@ -41704,7 +41454,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-2029-b59b-f9f9a653936a</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>1186</v>
       </c>
@@ -41727,7 +41477,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|019a8753-bf2c-6320-9905-6292b78d6e29</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>1187</v>
       </c>
@@ -41750,7 +41500,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|019a8753-bf2c-a49f-a4c9-d9396889bd0c</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>1188</v>
       </c>
@@ -41773,7 +41523,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|019a8753-bf2c-7967-8214-b5acd522f6a0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>1189</v>
       </c>
@@ -41796,7 +41546,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|019a8753-bf2c-f874-929d-fa14452a0de1</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>589</v>
       </c>
@@ -41819,7 +41569,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-a456-618e-e443bc0d35e9</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>590</v>
       </c>
@@ -41842,7 +41592,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-daa3-3b64-47a0bed70d1b</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>591</v>
       </c>
@@ -41865,7 +41615,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-7ab3-ba92-5fa2af40f240</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>592</v>
       </c>
@@ -41888,7 +41638,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-0e30-d86c-c2c7095525ec</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>593</v>
       </c>
@@ -41911,7 +41661,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-1443-43dc-7a07aef0da30</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>594</v>
       </c>
@@ -41934,7 +41684,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-7fbb-0745-44bb651edd00</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>595</v>
       </c>
@@ -41957,7 +41707,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-72db-d650-96776e8fd4a7</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>596</v>
       </c>
@@ -41980,7 +41730,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-aed3-82fc-8fc90e0c93fd</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>597</v>
       </c>
@@ -42003,7 +41753,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-e6af-3e5a-6494a01a06ae</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>598</v>
       </c>
@@ -42026,7 +41776,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-4e2b-87de-57604330cdd3</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>599</v>
       </c>
@@ -42049,7 +41799,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-7196-e13a-d911de7aa2aa</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>600</v>
       </c>
@@ -42072,7 +41822,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-49c9-f899-a2bd7ca7905e</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>601</v>
       </c>
@@ -42095,7 +41845,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-e911-0c7d-89e8d97702dc</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>602</v>
       </c>
@@ -42118,7 +41868,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-c287-9def-b1c31ccc15e3</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>603</v>
       </c>
@@ -42141,7 +41891,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-d41c-32e8-4166495e403d</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>604</v>
       </c>
@@ -42164,7 +41914,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-92f3-9168-2df7a147b28e</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>605</v>
       </c>
@@ -42187,7 +41937,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-83ae-9c38-8230890499d5</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>606</v>
       </c>
@@ -42210,7 +41960,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-aca5-d495-a14d205474c8</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>607</v>
       </c>
@@ -42233,7 +41983,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-059f-33dd-73f8668bc5ef</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>1190</v>
       </c>
@@ -42256,7 +42006,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|019a8753-bf2c-ac0e-6094-b453f8a8f0bf</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>1191</v>
       </c>
@@ -42279,7 +42029,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|019a8753-bf2c-72f3-1050-36bd41af94c6</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>1192</v>
       </c>
@@ -42302,7 +42052,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|019a8753-bf2c-9d55-e919-4048becd0188</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>1193</v>
       </c>
@@ -42325,7 +42075,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|019a8753-bf2c-31ce-e02e-41a60982d788</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>608</v>
       </c>
@@ -42348,7 +42098,7 @@
         <v>0195d18c-1cc1-44c2-1d6e-874dad333458|0198ef6d-8543-87f8-e4ed-200adf224eea</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>609</v>
       </c>
@@ -42371,7 +42121,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-a221-af7e-774497e4801a</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>610</v>
       </c>
@@ -42394,7 +42144,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-987d-80eb-fb29936d633c</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>611</v>
       </c>
@@ -42417,7 +42167,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-ce42-568c-c8e8405533a1</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>612</v>
       </c>
@@ -42440,7 +42190,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-8bc8-93ea-2f4c7e8626f2</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>613</v>
       </c>
@@ -42463,7 +42213,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-1062-3f54-74f967fd95da</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>614</v>
       </c>
@@ -42486,7 +42236,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-3bfd-fcb0-c5698a1b2d9a</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>615</v>
       </c>
@@ -42509,7 +42259,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-f372-ce25-38616e4c214d</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>616</v>
       </c>
@@ -42532,7 +42282,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-d9b1-6322-01cffb585d60</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>617</v>
       </c>
@@ -42555,7 +42305,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-b8fc-9de5-72be815082e0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>618</v>
       </c>
@@ -42578,7 +42328,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-f0ab-b028-4f183545ce97</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>619</v>
       </c>
@@ -42601,7 +42351,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-371a-179d-9c036f8c66f2</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>620</v>
       </c>
@@ -42624,7 +42374,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-7325-a3c3-0be3c6d6193b</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>621</v>
       </c>
@@ -42647,7 +42397,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-61b3-63f1-bc4f52741be3</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>622</v>
       </c>
@@ -42670,7 +42420,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-f6da-4821-571b2b52bd5b</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>623</v>
       </c>
@@ -42693,7 +42443,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-369f-5adc-42e8a92a03ef</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>624</v>
       </c>
@@ -42716,7 +42466,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-c2aa-d8d8-5799599aba32</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>625</v>
       </c>
@@ -42762,7 +42512,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-1f4a-69a6-ef2cbe30a080</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>627</v>
       </c>
@@ -42785,7 +42535,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-3dff-04fd-3c65614d655d</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>628</v>
       </c>
@@ -42808,7 +42558,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-c3d9-408d-20f86d523b9f</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>629</v>
       </c>
@@ -42831,7 +42581,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-e425-5793-c7c455726f56</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>630</v>
       </c>
@@ -42854,7 +42604,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-0bc5-2af0-dbe7f34bc5cc</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>631</v>
       </c>
@@ -42877,7 +42627,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-58d8-f78b-17d1fd52333b</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>632</v>
       </c>
@@ -42900,7 +42650,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-95f7-7801-f7b9a1173d31</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>633</v>
       </c>
@@ -42923,7 +42673,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-d942-891d-d90db771db73</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>634</v>
       </c>
@@ -42946,7 +42696,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-8e8e-2323-db15777c232c</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>635</v>
       </c>
@@ -42969,7 +42719,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-e881-c040-0a6a35d23358</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>636</v>
       </c>
@@ -42992,7 +42742,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-2162-0198-4b380cae3fa3</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>637</v>
       </c>
@@ -43015,7 +42765,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-f61d-4edc-07bcd51c380d</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>638</v>
       </c>
@@ -43038,7 +42788,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-6468-4596-cfc7b24c16e9</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>639</v>
       </c>
@@ -43061,7 +42811,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-2afc-2c12-93e895132544</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>640</v>
       </c>
@@ -43084,7 +42834,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-c453-7e15-c4a877df12b1</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>641</v>
       </c>
@@ -43107,7 +42857,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-2029-b59b-f9f9a653936a</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>642</v>
       </c>
@@ -43130,7 +42880,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-de89-1d51-d1a00a20cfe1</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>643</v>
       </c>
@@ -43153,7 +42903,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-2da2-cd65-fdc03f304e9b</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>644</v>
       </c>
@@ -43176,7 +42926,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-90ee-8214-09a6f499e9d9</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>1194</v>
       </c>
@@ -43199,7 +42949,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|019a8753-bf2c-ac0e-6094-b453f8a8f0bf</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>1195</v>
       </c>
@@ -43222,7 +42972,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|019a8753-bf2c-72f3-1050-36bd41af94c6</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>1196</v>
       </c>
@@ -43245,7 +42995,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|019a8753-bf2c-9d55-e919-4048becd0188</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>1197</v>
       </c>
@@ -43268,7 +43018,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|019a8753-bf2c-31ce-e02e-41a60982d788</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>1198</v>
       </c>
@@ -43291,7 +43041,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|019a8753-bf2c-631f-91f0-cd8c0742426e</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>1199</v>
       </c>
@@ -43314,7 +43064,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|019a8753-bf2c-e119-fd51-451b080ba5e2</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>1200</v>
       </c>
@@ -43337,7 +43087,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|019a8753-bf2c-c21b-8e4c-6a7c42d05ab8</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>1201</v>
       </c>
@@ -43360,7 +43110,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|019a8753-bf2c-eaec-ad1a-19099112f11b</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>645</v>
       </c>
@@ -43383,7 +43133,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-a456-618e-e443bc0d35e9</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>646</v>
       </c>
@@ -43406,7 +43156,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-5532-be80-6c8a18c388da</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>647</v>
       </c>
@@ -43429,7 +43179,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-daa3-3b64-47a0bed70d1b</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>648</v>
       </c>
@@ -43452,7 +43202,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-7ab3-ba92-5fa2af40f240</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>649</v>
       </c>
@@ -43475,7 +43225,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-0e30-d86c-c2c7095525ec</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>650</v>
       </c>
@@ -43498,7 +43248,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-1443-43dc-7a07aef0da30</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>651</v>
       </c>
@@ -43521,7 +43271,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-7fbb-0745-44bb651edd00</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>652</v>
       </c>
@@ -43544,7 +43294,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-72db-d650-96776e8fd4a7</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>653</v>
       </c>
@@ -43567,7 +43317,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-aed3-82fc-8fc90e0c93fd</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>654</v>
       </c>
@@ -43590,7 +43340,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-e6af-3e5a-6494a01a06ae</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>655</v>
       </c>
@@ -43613,7 +43363,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-4e2b-87de-57604330cdd3</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>656</v>
       </c>
@@ -43636,7 +43386,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-7196-e13a-d911de7aa2aa</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>657</v>
       </c>
@@ -43659,7 +43409,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-49c9-f899-a2bd7ca7905e</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>658</v>
       </c>
@@ -43682,7 +43432,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-e911-0c7d-89e8d97702dc</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>659</v>
       </c>
@@ -43705,7 +43455,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-c287-9def-b1c31ccc15e3</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>660</v>
       </c>
@@ -43728,7 +43478,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-d41c-32e8-4166495e403d</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>661</v>
       </c>
@@ -43751,7 +43501,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-92f3-9168-2df7a147b28e</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>662</v>
       </c>
@@ -43774,7 +43524,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-83ae-9c38-8230890499d5</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>663</v>
       </c>
@@ -43797,7 +43547,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-aca5-d495-a14d205474c8</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>664</v>
       </c>
@@ -43820,7 +43570,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|0198ef6d-8543-059f-33dd-73f8668bc5ef</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>1202</v>
       </c>
@@ -43843,7 +43593,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|019a8753-bf2c-ac0e-6094-b453f8a8f0bf</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>1203</v>
       </c>
@@ -43866,7 +43616,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|019a8753-bf2c-72f3-1050-36bd41af94c6</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>1204</v>
       </c>
@@ -43889,7 +43639,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|019a8753-bf2c-9d55-e919-4048becd0188</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>1205</v>
       </c>
@@ -43912,7 +43662,7 @@
         <v>0195d18c-1cc1-c475-eba4-c3df5aea8858|019a8753-bf2c-31ce-e02e-41a60982d788</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>665</v>
       </c>
@@ -43936,7 +43686,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H116" xr:uid="{00000000-0001-0000-0800-000000000000}"/>
+  <autoFilter ref="A1:H116" xr:uid="{00000000-0001-0000-0800-000000000000}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="0198ef6d-8543-1f4a-69a6-ef2cbe30a080"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -44216,18 +43972,18 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>64</v>
+        <v>132</v>
       </c>
       <c r="K2" s="4" t="str">
         <f>IF($J2="","",INDEX(CaseTypeColSet!$B:$B,MATCH($J2,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1</v>
+        <v>case_type_col_set1_1and2</v>
       </c>
       <c r="L2" t="s">
-        <v>64</v>
+        <v>132</v>
       </c>
       <c r="M2" s="4" t="str">
         <f>IF($L2="","",INDEX(CaseTypeColSet!$B:$B,MATCH($L2,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1</v>
+        <v>case_type_col_set1_1and2</v>
       </c>
       <c r="N2" t="b">
         <v>1</v>
@@ -44669,11 +44425,11 @@
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="K8" s="4" t="str">
         <f>IF($J8="","",INDEX(CaseTypeColSet!$B:$B,MATCH($J8,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1and2</v>
+        <v>case_type_col_set1_1</v>
       </c>
       <c r="M8" s="4" t="str">
         <f>IF($L8="","",INDEX(CaseTypeColSet!$B:$B,MATCH($L8,CaseTypeColSet!$A:$A,0)))</f>
@@ -44742,11 +44498,11 @@
         <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="K9" s="4" t="str">
         <f>IF($J9="","",INDEX(CaseTypeColSet!$B:$B,MATCH($J9,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1and2</v>
+        <v>case_type_col_set1_1</v>
       </c>
       <c r="M9" s="4" t="str">
         <f>IF($L9="","",INDEX(CaseTypeColSet!$B:$B,MATCH($L9,CaseTypeColSet!$A:$A,0)))</f>
@@ -44815,11 +44571,11 @@
         <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="K10" s="4" t="str">
         <f>IF($J10="","",INDEX(CaseTypeColSet!$B:$B,MATCH($J10,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1and2</v>
+        <v>case_type_col_set1_1</v>
       </c>
       <c r="M10" s="4" t="str">
         <f>IF($L10="","",INDEX(CaseTypeColSet!$B:$B,MATCH($L10,CaseTypeColSet!$A:$A,0)))</f>
@@ -44888,11 +44644,11 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="K11" s="4" t="str">
         <f>IF($J11="","",INDEX(CaseTypeColSet!$B:$B,MATCH($J11,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1and2</v>
+        <v>case_type_col_set1_1</v>
       </c>
       <c r="M11" s="4" t="str">
         <f>IF($L11="","",INDEX(CaseTypeColSet!$B:$B,MATCH($L11,CaseTypeColSet!$A:$A,0)))</f>
@@ -45063,18 +44819,18 @@
         <v>1</v>
       </c>
       <c r="I2" t="s">
-        <v>64</v>
+        <v>132</v>
       </c>
       <c r="J2" s="4" t="str">
         <f>IF($I2="","",INDEX(CaseTypeColSet!$B:$B,MATCH($I2,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1</v>
+        <v>case_type_col_set1_1and2</v>
       </c>
       <c r="K2" t="s">
-        <v>64</v>
+        <v>132</v>
       </c>
       <c r="L2" s="4" t="str">
         <f>IF($K2="","",INDEX(CaseTypeColSet!$B:$B,MATCH($K2,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1</v>
+        <v>case_type_col_set1_1and2</v>
       </c>
       <c r="M2" t="b">
         <v>1</v>
@@ -45549,18 +45305,18 @@
         <v>1</v>
       </c>
       <c r="I8" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="J8" s="4" t="str">
         <f>IF($I8="","",INDEX(CaseTypeColSet!$B:$B,MATCH($I8,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1and2</v>
+        <v>case_type_col_set1_1</v>
       </c>
       <c r="K8" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="L8" s="4" t="str">
         <f>IF($K8="","",INDEX(CaseTypeColSet!$B:$B,MATCH($K8,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1and2</v>
+        <v>case_type_col_set1_1</v>
       </c>
       <c r="M8" t="b">
         <v>1</v>
@@ -45630,18 +45386,18 @@
         <v>1</v>
       </c>
       <c r="I9" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="J9" s="4" t="str">
         <f>IF($I9="","",INDEX(CaseTypeColSet!$B:$B,MATCH($I9,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1and2</v>
+        <v>case_type_col_set1_1</v>
       </c>
       <c r="K9" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="L9" s="4" t="str">
         <f>IF($K9="","",INDEX(CaseTypeColSet!$B:$B,MATCH($K9,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1and2</v>
+        <v>case_type_col_set1_1</v>
       </c>
       <c r="M9" t="b">
         <v>1</v>
@@ -45711,18 +45467,18 @@
         <v>1</v>
       </c>
       <c r="I10" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="J10" s="4" t="str">
         <f>IF($I10="","",INDEX(CaseTypeColSet!$B:$B,MATCH($I10,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1and2</v>
+        <v>case_type_col_set1_1</v>
       </c>
       <c r="K10" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="L10" s="4" t="str">
         <f>IF($K10="","",INDEX(CaseTypeColSet!$B:$B,MATCH($K10,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1and2</v>
+        <v>case_type_col_set1_1</v>
       </c>
       <c r="M10" t="b">
         <v>1</v>
@@ -45792,18 +45548,18 @@
         <v>1</v>
       </c>
       <c r="I11" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="J11" s="4" t="str">
         <f>IF($I11="","",INDEX(CaseTypeColSet!$B:$B,MATCH($I11,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1and2</v>
+        <v>case_type_col_set1_1</v>
       </c>
       <c r="K11" t="s">
-        <v>132</v>
+        <v>64</v>
       </c>
       <c r="L11" s="4" t="str">
         <f>IF($K11="","",INDEX(CaseTypeColSet!$B:$B,MATCH($K11,CaseTypeColSet!$A:$A,0)))</f>
-        <v>case_type_col_set1_1and2</v>
+        <v>case_type_col_set1_1</v>
       </c>
       <c r="M11" t="b">
         <v>1</v>

</xml_diff>